<commit_message>
feat: end-to-end pipeline runs clean (all 4 models + fusion) + cleanup stale docs
Pipeline now wired end-to-end through main.py -> staged_pipeline.py:

- All 4 model pipelines (SGDFNet, TimeMixer, RT916, TimesFM) + fusion are runnable from a single entrypoint

- Update data: data/shandong_pmos_hourly.{csv,xlsx}, ExtremPriceClf/data/*, add data/p1交割概览/p1.xlsx

- Add helper scripts: _calc_metrics.py, _inspect_excel.py

- Add optim/ module (perf knobs, init) for the new pipeline

- Update core: cli/parser.py, main.py, pipelines/staged_pipeline.py, fusion/*, TimeMixer/{pipeline,repro_pipeline}.py, RT916_SpikeFusionNet/{pipeline,src/core}.py, SGDFNet/pipeline.py, requirements.txt, README.md

- Remove 33 stale docs: FUSION_V1_*, MEMORY.md, PROJECT_ENTRYPOINTS.md, all codex_prompt_*, Codex执行*, TimeMixer收尾/审计/出区/计算/当前总结, SGDFNet审计, AMP_DataLoader_TF32, 三大训练加速, 分类器集成, 收尾与训练优化, 清理收尾与下一, 承袭链路TimesFM回填, 计算毕评估, 项目封装与统一运行重构, 项目清理与补全
</commit_message>
<xml_diff>
--- a/ExtremPriceClf/data/融合模型预测电价数据.xlsx
+++ b/ExtremPriceClf/data/融合模型预测电价数据.xlsx
@@ -377,7 +377,7 @@
         <v>46157.04166666666</v>
       </c>
       <c r="B2">
-        <v>527.5861672886069</v>
+        <v>322.1432743580563</v>
       </c>
       <c r="C2">
         <v>495.652</v>
@@ -388,7 +388,7 @@
         <v>46157.08333333334</v>
       </c>
       <c r="B3">
-        <v>496.4285510670013</v>
+        <v>318.6418092410445</v>
       </c>
       <c r="C3">
         <v>446.483</v>
@@ -399,7 +399,7 @@
         <v>46157.125</v>
       </c>
       <c r="B4">
-        <v>474.5993021730459</v>
+        <v>285.6717564995837</v>
       </c>
       <c r="C4">
         <v>411.384</v>
@@ -410,7 +410,7 @@
         <v>46157.16666666666</v>
       </c>
       <c r="B5">
-        <v>476.8284074961273</v>
+        <v>318.6418092410445</v>
       </c>
       <c r="C5">
         <v>409.424</v>
@@ -421,7 +421,7 @@
         <v>46157.20833333334</v>
       </c>
       <c r="B6">
-        <v>499.2816225965585</v>
+        <v>322.1432743580563</v>
       </c>
       <c r="C6">
         <v>432.173</v>
@@ -432,7 +432,7 @@
         <v>46157.25</v>
       </c>
       <c r="B7">
-        <v>524.3633591269712</v>
+        <v>322.1432743580563</v>
       </c>
       <c r="C7">
         <v>451.669</v>
@@ -443,7 +443,7 @@
         <v>46157.29166666666</v>
       </c>
       <c r="B8">
-        <v>320.2652232612188</v>
+        <v>226.3296484182191</v>
       </c>
       <c r="C8">
         <v>471.098</v>
@@ -454,7 +454,7 @@
         <v>46157.33333333334</v>
       </c>
       <c r="B9">
-        <v>-46.20590232878574</v>
+        <v>192.7170787192855</v>
       </c>
       <c r="C9">
         <v>453.471</v>
@@ -465,7 +465,7 @@
         <v>46157.375</v>
       </c>
       <c r="B10">
-        <v>43.64623242480774</v>
+        <v>-71.75950548749653</v>
       </c>
       <c r="C10">
         <v>554.0119999999999</v>
@@ -476,7 +476,7 @@
         <v>46157.41666666666</v>
       </c>
       <c r="B11">
-        <v>-82.46291932801699</v>
+        <v>-71.51409217540287</v>
       </c>
       <c r="C11">
         <v>114.886</v>
@@ -487,7 +487,7 @@
         <v>46157.45833333334</v>
       </c>
       <c r="B12">
-        <v>-99.6588795957538</v>
+        <v>-69.37335619969566</v>
       </c>
       <c r="C12">
         <v>-73.846</v>
@@ -498,7 +498,7 @@
         <v>46157.5</v>
       </c>
       <c r="B13">
-        <v>-122.3441226565707</v>
+        <v>-68.13762650307268</v>
       </c>
       <c r="C13">
         <v>-73.08199999999999</v>
@@ -509,7 +509,7 @@
         <v>46157.54166666666</v>
       </c>
       <c r="B14">
-        <v>-147.8060758386412</v>
+        <v>-68.09915425438</v>
       </c>
       <c r="C14">
         <v>-59.314</v>
@@ -520,7 +520,7 @@
         <v>46157.58333333334</v>
       </c>
       <c r="B15">
-        <v>-121.9801765436098</v>
+        <v>-68.65389790855798</v>
       </c>
       <c r="C15">
         <v>-62.831</v>
@@ -531,7 +531,7 @@
         <v>46157.625</v>
       </c>
       <c r="B16">
-        <v>-86.51583540805568</v>
+        <v>-71.02724114207852</v>
       </c>
       <c r="C16">
         <v>-76.89700000000001</v>
@@ -542,7 +542,7 @@
         <v>46157.66666666666</v>
       </c>
       <c r="B17">
-        <v>22.70859964916107</v>
+        <v>-74.61032600112701</v>
       </c>
       <c r="C17">
         <v>-31</v>
@@ -553,7 +553,7 @@
         <v>46157.70833333334</v>
       </c>
       <c r="B18">
-        <v>311.6561421110388</v>
+        <v>113.840281954686</v>
       </c>
       <c r="C18">
         <v>392.751</v>
@@ -564,7 +564,7 @@
         <v>46157.75</v>
       </c>
       <c r="B19">
-        <v>471.5587023257037</v>
+        <v>354.9521338102093</v>
       </c>
       <c r="C19">
         <v>601.99</v>
@@ -575,7 +575,7 @@
         <v>46157.79166666666</v>
       </c>
       <c r="B20">
-        <v>536.4536068514127</v>
+        <v>429.1054515349668</v>
       </c>
       <c r="C20">
         <v>611.1609999999999</v>
@@ -586,7 +586,7 @@
         <v>46157.83333333334</v>
       </c>
       <c r="B21">
-        <v>556.5017017946619</v>
+        <v>510.8302738517863</v>
       </c>
       <c r="C21">
         <v>593.246</v>
@@ -597,7 +597,7 @@
         <v>46157.875</v>
       </c>
       <c r="B22">
-        <v>546.5591429188446</v>
+        <v>520.6495788484577</v>
       </c>
       <c r="C22">
         <v>585.47</v>
@@ -608,7 +608,7 @@
         <v>46157.91666666666</v>
       </c>
       <c r="B23">
-        <v>549.3236164554747</v>
+        <v>528.0390535379938</v>
       </c>
       <c r="C23">
         <v>586.4299999999999</v>
@@ -619,7 +619,7 @@
         <v>46157.95833333334</v>
       </c>
       <c r="B24">
-        <v>532.1104025077099</v>
+        <v>475.3991851022369</v>
       </c>
       <c r="C24">
         <v>615.519</v>
@@ -630,7 +630,7 @@
         <v>46158</v>
       </c>
       <c r="B25">
-        <v>39.14337251165242</v>
+        <v>332.4705170424747</v>
       </c>
       <c r="C25">
         <v>581.543</v>

</xml_diff>

<commit_message>
fix(RT916): disable AMP during inference to avoid BFloat16->numpy dtype error
- RT916 weights are saved in BFloat16; numpy cannot convert them, so inference must run with OPTIM_AMP=0

- Training still benefits from AMP (separate code path)

- Remove _calc_metrics.py and _inspect_excel.py (consolidated into optim/perf_knobs.py and main entrypoint)

- Refresh data snapshots: ExtremPriceClf/data/p1交割概览/p1.xlsx, ExtremPriceClf/data/承袭模型预测电价数据.xlsx
</commit_message>
<xml_diff>
--- a/ExtremPriceClf/data/融合模型预测电价数据.xlsx
+++ b/ExtremPriceClf/data/融合模型预测电价数据.xlsx
@@ -374,266 +374,266 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1">
-        <v>46157.04166666666</v>
+        <v>46162.04166666666</v>
       </c>
       <c r="B2">
-        <v>322.1432743580563</v>
+        <v>340.1705357103355</v>
       </c>
       <c r="C2">
-        <v>495.652</v>
+        <v>312.967</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1">
-        <v>46157.08333333334</v>
+        <v>46162.08333333334</v>
       </c>
       <c r="B3">
-        <v>318.6418092410445</v>
+        <v>326.2069040753889</v>
       </c>
       <c r="C3">
-        <v>446.483</v>
+        <v>302.863</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1">
-        <v>46157.125</v>
+        <v>46162.125</v>
       </c>
       <c r="B4">
-        <v>285.6717564995837</v>
+        <v>311.3104648621803</v>
       </c>
       <c r="C4">
-        <v>411.384</v>
+        <v>263.465</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1">
-        <v>46157.16666666666</v>
+        <v>46162.16666666666</v>
       </c>
       <c r="B5">
-        <v>318.6418092410445</v>
+        <v>311.7822215834518</v>
       </c>
       <c r="C5">
-        <v>409.424</v>
+        <v>210.342</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1">
-        <v>46157.20833333334</v>
+        <v>46162.20833333334</v>
       </c>
       <c r="B6">
-        <v>322.1432743580563</v>
+        <v>315.810881316071</v>
       </c>
       <c r="C6">
-        <v>432.173</v>
+        <v>222.744</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1">
-        <v>46157.25</v>
+        <v>46162.25</v>
       </c>
       <c r="B7">
-        <v>322.1432743580563</v>
+        <v>317.8747313254686</v>
       </c>
       <c r="C7">
-        <v>451.669</v>
+        <v>275.429</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1">
-        <v>46157.29166666666</v>
+        <v>46162.29166666666</v>
       </c>
       <c r="B8">
-        <v>226.3296484182191</v>
+        <v>290.6889805968045</v>
       </c>
       <c r="C8">
-        <v>471.098</v>
+        <v>317.004</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1">
-        <v>46157.33333333334</v>
+        <v>46162.33333333334</v>
       </c>
       <c r="B9">
-        <v>192.7170787192855</v>
+        <v>320.4382014742271</v>
       </c>
       <c r="C9">
-        <v>453.471</v>
+        <v>384.536</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1">
-        <v>46157.375</v>
+        <v>46162.375</v>
       </c>
       <c r="B10">
-        <v>-71.75950548749653</v>
+        <v>-7.998269419181796</v>
       </c>
       <c r="C10">
-        <v>554.0119999999999</v>
+        <v>461.913</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1">
-        <v>46157.41666666666</v>
+        <v>46162.41666666666</v>
       </c>
       <c r="B11">
-        <v>-71.51409217540287</v>
+        <v>-33.69076398553986</v>
       </c>
       <c r="C11">
-        <v>114.886</v>
+        <v>476.588</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1">
-        <v>46157.45833333334</v>
+        <v>46162.45833333334</v>
       </c>
       <c r="B12">
-        <v>-69.37335619969566</v>
+        <v>-65.28945958052985</v>
       </c>
       <c r="C12">
-        <v>-73.846</v>
+        <v>497.088</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1">
-        <v>46157.5</v>
+        <v>46162.5</v>
       </c>
       <c r="B13">
-        <v>-68.13762650307268</v>
+        <v>-71.29639581352538</v>
       </c>
       <c r="C13">
-        <v>-73.08199999999999</v>
+        <v>499.936</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1">
-        <v>46157.54166666666</v>
+        <v>46162.54166666666</v>
       </c>
       <c r="B14">
-        <v>-68.09915425438</v>
+        <v>-47.00193608413782</v>
       </c>
       <c r="C14">
-        <v>-59.314</v>
+        <v>454.932</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1">
-        <v>46157.58333333334</v>
+        <v>46162.58333333334</v>
       </c>
       <c r="B15">
-        <v>-68.65389790855798</v>
+        <v>-32.99732674295728</v>
       </c>
       <c r="C15">
-        <v>-62.831</v>
+        <v>440.991</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1">
-        <v>46157.625</v>
+        <v>46162.625</v>
       </c>
       <c r="B16">
-        <v>-71.02724114207852</v>
+        <v>-31.02262696362391</v>
       </c>
       <c r="C16">
-        <v>-76.89700000000001</v>
+        <v>415.458</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1">
-        <v>46157.66666666666</v>
+        <v>46162.66666666666</v>
       </c>
       <c r="B17">
-        <v>-74.61032600112701</v>
+        <v>-39.73383687083712</v>
       </c>
       <c r="C17">
-        <v>-31</v>
+        <v>359.168</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1">
-        <v>46157.70833333334</v>
+        <v>46162.70833333334</v>
       </c>
       <c r="B18">
-        <v>113.840281954686</v>
+        <v>349.3163127662976</v>
       </c>
       <c r="C18">
-        <v>392.751</v>
+        <v>375.89</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1">
-        <v>46157.75</v>
+        <v>46162.75</v>
       </c>
       <c r="B19">
-        <v>354.9521338102093</v>
+        <v>364.9618387978657</v>
       </c>
       <c r="C19">
-        <v>601.99</v>
+        <v>327.262</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1">
-        <v>46157.79166666666</v>
+        <v>46162.79166666666</v>
       </c>
       <c r="B20">
-        <v>429.1054515349668</v>
+        <v>402.1305838609725</v>
       </c>
       <c r="C20">
-        <v>611.1609999999999</v>
+        <v>404.043</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1">
-        <v>46157.83333333334</v>
+        <v>46162.83333333334</v>
       </c>
       <c r="B21">
-        <v>510.8302738517863</v>
+        <v>424.6128933776117</v>
       </c>
       <c r="C21">
-        <v>593.246</v>
+        <v>440.832</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1">
-        <v>46157.875</v>
+        <v>46162.875</v>
       </c>
       <c r="B22">
-        <v>520.6495788484577</v>
+        <v>424.5858968743472</v>
       </c>
       <c r="C22">
-        <v>585.47</v>
+        <v>420.1</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1">
-        <v>46157.91666666666</v>
+        <v>46162.91666666666</v>
       </c>
       <c r="B23">
-        <v>528.0390535379938</v>
+        <v>428.5230364976271</v>
       </c>
       <c r="C23">
-        <v>586.4299999999999</v>
+        <v>381.371</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1">
-        <v>46157.95833333334</v>
+        <v>46162.95833333334</v>
       </c>
       <c r="B24">
-        <v>475.3991851022369</v>
+        <v>436.568268274618</v>
       </c>
       <c r="C24">
-        <v>615.519</v>
+        <v>396.961</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1">
-        <v>46158</v>
+        <v>46163</v>
       </c>
       <c r="B25">
-        <v>332.4705170424747</v>
+        <v>413.7807105280298</v>
       </c>
       <c r="C25">
-        <v>581.543</v>
+        <v>370.492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: one-command full pipeline + fix model path issues + update docs
- Add `python main.py <DATE>` shortcut for full 4-stage pipeline
  (model_stage → learner_stage → fuse_stage → classifier_stage)
- Fix RT916: override frozen core.RAW_DF_PATH before calling core functions
- Fix TimeMixer: replace hardcoded absolute paths with relative Path(__file__)
- Fix TimesFM: raise RuntimeError when model weights missing (was silent skip)
- Fix staged_pipeline: add model status tracking, non-empty CSV check, summary log
- Fix executor: log warning when model returns None
- Fix LightGBM: replace print with logger.error in exception handlers
- Update README: add TimesFM weight download instructions, one-command usage,
  reproducibility checklist, updated CLI parameter table
- Update requirements.txt: clean up dependencies, mark Flax stack as optional
- Update .gitignore: exclude daily_runs_*/ and ad-hoc scripts
</commit_message>
<xml_diff>
--- a/ExtremPriceClf/data/融合模型预测电价数据.xlsx
+++ b/ExtremPriceClf/data/融合模型预测电价数据.xlsx
@@ -374,266 +374,266 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1">
-        <v>46162.04166666666</v>
+        <v>46054.04166666666</v>
       </c>
       <c r="B2">
-        <v>340.1705357103355</v>
+        <v>378.962658331683</v>
       </c>
       <c r="C2">
-        <v>312.967</v>
+        <v>376.978</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1">
-        <v>46162.08333333334</v>
+        <v>46054.08333333334</v>
       </c>
       <c r="B3">
-        <v>326.2069040753889</v>
+        <v>362.1687235098425</v>
       </c>
       <c r="C3">
-        <v>302.863</v>
+        <v>353.014</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1">
-        <v>46162.125</v>
+        <v>46054.125</v>
       </c>
       <c r="B4">
-        <v>311.3104648621803</v>
+        <v>377.4782350404463</v>
       </c>
       <c r="C4">
-        <v>263.465</v>
+        <v>364.613</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1">
-        <v>46162.16666666666</v>
+        <v>46054.16666666666</v>
       </c>
       <c r="B5">
-        <v>311.7822215834518</v>
+        <v>355.1267072163429</v>
       </c>
       <c r="C5">
-        <v>210.342</v>
+        <v>347.423</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1">
-        <v>46162.20833333334</v>
+        <v>46054.20833333334</v>
       </c>
       <c r="B6">
-        <v>315.810881316071</v>
+        <v>351.5305889210525</v>
       </c>
       <c r="C6">
-        <v>222.744</v>
+        <v>340.032</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1">
-        <v>46162.25</v>
+        <v>46054.25</v>
       </c>
       <c r="B7">
-        <v>317.8747313254686</v>
+        <v>312.1166659245042</v>
       </c>
       <c r="C7">
-        <v>275.429</v>
+        <v>307.932</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1">
-        <v>46162.29166666666</v>
+        <v>46054.29166666666</v>
       </c>
       <c r="B8">
-        <v>290.6889805968045</v>
+        <v>282.0537338297029</v>
       </c>
       <c r="C8">
-        <v>317.004</v>
+        <v>196.874</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1">
-        <v>46162.33333333334</v>
+        <v>46054.33333333334</v>
       </c>
       <c r="B9">
-        <v>320.4382014742271</v>
+        <v>321.3456329799322</v>
       </c>
       <c r="C9">
-        <v>384.536</v>
+        <v>356.643</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1">
-        <v>46162.375</v>
+        <v>46054.375</v>
       </c>
       <c r="B10">
-        <v>-7.998269419181796</v>
+        <v>268.8118315508629</v>
       </c>
       <c r="C10">
-        <v>461.913</v>
+        <v>400.267</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1">
-        <v>46162.41666666666</v>
+        <v>46054.41666666666</v>
       </c>
       <c r="B11">
-        <v>-33.69076398553986</v>
+        <v>65.75864592376783</v>
       </c>
       <c r="C11">
-        <v>476.588</v>
+        <v>432.641</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1">
-        <v>46162.45833333334</v>
+        <v>46054.45833333334</v>
       </c>
       <c r="B12">
-        <v>-65.28945958052985</v>
+        <v>-17.17883441107117</v>
       </c>
       <c r="C12">
-        <v>497.088</v>
+        <v>456.179</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1">
-        <v>46162.5</v>
+        <v>46054.5</v>
       </c>
       <c r="B13">
-        <v>-71.29639581352538</v>
+        <v>-14.54635063131135</v>
       </c>
       <c r="C13">
-        <v>499.936</v>
+        <v>469.704</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1">
-        <v>46162.54166666666</v>
+        <v>46054.54166666666</v>
       </c>
       <c r="B14">
-        <v>-47.00193608413782</v>
+        <v>-55.38294020382369</v>
       </c>
       <c r="C14">
-        <v>454.932</v>
+        <v>435.397</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1">
-        <v>46162.58333333334</v>
+        <v>46054.58333333334</v>
       </c>
       <c r="B15">
-        <v>-32.99732674295728</v>
+        <v>-45.04168233807954</v>
       </c>
       <c r="C15">
-        <v>440.991</v>
+        <v>382.755</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1">
-        <v>46162.625</v>
+        <v>46054.625</v>
       </c>
       <c r="B16">
-        <v>-31.02262696362391</v>
+        <v>61.79626179629913</v>
       </c>
       <c r="C16">
-        <v>415.458</v>
+        <v>350.422</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1">
-        <v>46162.66666666666</v>
+        <v>46054.66666666666</v>
       </c>
       <c r="B17">
-        <v>-39.73383687083712</v>
+        <v>178.1145100459733</v>
       </c>
       <c r="C17">
-        <v>359.168</v>
+        <v>376.177</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1">
-        <v>46162.70833333334</v>
+        <v>46054.70833333334</v>
       </c>
       <c r="B18">
-        <v>349.3163127662976</v>
+        <v>342.0738131709059</v>
       </c>
       <c r="C18">
-        <v>375.89</v>
+        <v>429.143</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1">
-        <v>46162.75</v>
+        <v>46054.75</v>
       </c>
       <c r="B19">
-        <v>364.9618387978657</v>
+        <v>368.5097345617228</v>
       </c>
       <c r="C19">
-        <v>327.262</v>
+        <v>437.715</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1">
-        <v>46162.79166666666</v>
+        <v>46054.79166666666</v>
       </c>
       <c r="B20">
-        <v>402.1305838609725</v>
+        <v>355.0577140366143</v>
       </c>
       <c r="C20">
-        <v>404.043</v>
+        <v>441.233</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1">
-        <v>46162.83333333334</v>
+        <v>46054.83333333334</v>
       </c>
       <c r="B21">
-        <v>424.6128933776117</v>
+        <v>346.8859176692166</v>
       </c>
       <c r="C21">
-        <v>440.832</v>
+        <v>437.852</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1">
-        <v>46162.875</v>
+        <v>46054.875</v>
       </c>
       <c r="B22">
-        <v>424.5858968743472</v>
+        <v>341.6233922645597</v>
       </c>
       <c r="C22">
-        <v>420.1</v>
+        <v>445.232</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1">
-        <v>46162.91666666666</v>
+        <v>46054.91666666666</v>
       </c>
       <c r="B23">
-        <v>428.5230364976271</v>
+        <v>345.5806188802712</v>
       </c>
       <c r="C23">
-        <v>381.371</v>
+        <v>444.737</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1">
-        <v>46162.95833333334</v>
+        <v>46054.95833333334</v>
       </c>
       <c r="B24">
-        <v>436.568268274618</v>
+        <v>354.955019960005</v>
       </c>
       <c r="C24">
-        <v>396.961</v>
+        <v>430.964</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1">
-        <v>46163</v>
+        <v>46055</v>
       </c>
       <c r="B25">
-        <v>413.7807105280298</v>
+        <v>381.6441209806853</v>
       </c>
       <c r="C25">
-        <v>370.492</v>
+        <v>425.109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>